<commit_message>
docs: update test report to 60 tests
</commit_message>
<xml_diff>
--- a/doc/test-report.xlsx
+++ b/doc/test-report.xlsx
@@ -13,9 +13,9 @@
     <sheet name="รายละเอียดเทสเคส" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">รายละเอียดเทสเคส!$A$1:$F$58</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">รายละเอียดเทสเคส!$A$1:$F$60</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr fullCalcOnLoad="1" iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -42,7 +42,7 @@
     <t xml:space="preserve">ขอบเขตการทดสอบ</t>
   </si>
   <si>
-    <t xml:space="preserve">6 คลาส: Member, Membership, MembershipPlan, Trainer, MemberInfo, TrainingSession (ไฟล์ *ServiceImplTest) รวม 57 เทสเคส</t>
+    <t xml:space="preserve">6 คลาส: Member, Membership, MembershipPlan, Trainer, MemberInfo, TrainingSession (ไฟล์ *ServiceImplTest) รวม 59 เทสเคส</t>
   </si>
   <si>
     <t xml:space="preserve">วิธีการทดสอบ</t>
@@ -78,13 +78,13 @@
     <t xml:space="preserve">ผลโดยรวม</t>
   </si>
   <si>
-    <t xml:space="preserve">BUILD SUCCESS — ผ่าน 57 จาก 57 เทสเคส (รายละเอียดดูชีต "สรุปผล")</t>
+    <t xml:space="preserve">BUILD SUCCESS — ผ่าน 59 จาก 59 เทสเคส (รายละเอียดดูชีต "สรุปผล")</t>
   </si>
   <si>
     <t xml:space="preserve">หมายเหตุ</t>
   </si>
   <si>
-    <t xml:space="preserve">การรัน ./mvnw test ทั้งโปรเจกต์ จะมี MembershipApplicationTests (ตรวจว่า Spring context บูตและต่อ DB ได้) เพิ่มอีก 1 เทสต์ รวมเป็น 58 รายงานนี้นับเฉพาะ 57 เทสเคสของ service</t>
+    <t xml:space="preserve">การรัน ./mvnw test ทั้งโปรเจกต์ จะมี MembershipApplicationTests (ตรวจว่า Spring context บูตและต่อ DB ได้) เพิ่มอีก 1 เทสต์ รวมเป็น 60 รายงานนี้นับเฉพาะ 59 เทสเคสของ service</t>
   </si>
   <si>
     <t xml:space="preserve">แท็บในไฟล์นี้</t>
@@ -99,7 +99,7 @@
     <t xml:space="preserve">รายละเอียดเทสเคส</t>
   </si>
   <si>
-    <t xml:space="preserve">รายการเทสเคสทั้ง 57 ข้อ พร้อม Test ID คลาส ชื่อ method ผลลัพธ์ และประเภทเทสต์</t>
+    <t xml:space="preserve">รายการเทสเคสทั้ง 59 ข้อ พร้อม Test ID คลาส ชื่อ method ผลลัพธ์ และประเภทเทสต์</t>
   </si>
   <si>
     <t xml:space="preserve">สรุปผลการทดสอบ</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">หมายเหตุ: ตัวเลขสีน้ำเงิน (เวลา) คัดจาก log การรัน Maven ของคลาสนั้นโดยตรง ส่วนจำนวนเทสต์/ผ่าน/ไม่ผ่านคำนวณจากชีต "รายละเอียดเทสเคส"</t>
   </si>
   <si>
-    <t xml:space="preserve">ผลโดยรวมจาก Maven: BUILD SUCCESS, Tests run: 57, Failures: 0, Errors: 0, Skipped: 0</t>
+    <t xml:space="preserve">ผลโดยรวมจาก Maven: BUILD SUCCESS, Tests run: 59, Failures: 0, Errors: 0, Skipped: 0</t>
   </si>
   <si>
     <t xml:space="preserve">Test ID</t>
@@ -1147,7 +1147,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>14</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>9</c:v>
@@ -1488,7 +1488,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>57</c:v>
+                  <c:v>59</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1680,22 +1680,22 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.549</c:v>
+                  <c:v>0.607</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.063</c:v>
+                  <c:v>0.059</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.016</c:v>
+                  <c:v>0.018</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.02</c:v>
+                  <c:v>0.019</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.026</c:v>
+                  <c:v>0.023</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.04</c:v>
+                  <c:v>0.018</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2243,8 +2243,8 @@
         <v>26</v>
       </c>
       <c r="B3" s="9" t="n">
-        <f aca="false">COUNTA(รายละเอียดเทสเคส!A2:A58)</f>
-        <v>57</v>
+        <f aca="false">COUNTA(รายละเอียดเทสเคส!A2:A60)</f>
+        <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2252,8 +2252,8 @@
         <v>27</v>
       </c>
       <c r="B4" s="10" t="n">
-        <f aca="false">COUNTIF(รายละเอียดเทสเคส!E2:E58,"PASS")</f>
-        <v>57</v>
+        <f aca="false">COUNTIF(รายละเอียดเทสเคส!E2:E60,"PASS")</f>
+        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2261,7 +2261,7 @@
         <v>28</v>
       </c>
       <c r="B5" s="9" t="n">
-        <f aca="false">COUNTIF(รายละเอียดเทสเคส!E2:E58,"FAIL")</f>
+        <f aca="false">COUNTIF(รายละเอียดเทสเคส!E2:E60,"FAIL")</f>
         <v>0</v>
       </c>
     </row>
@@ -2302,12 +2302,12 @@
         <v>34</v>
       </c>
       <c r="B10" s="14" t="n">
-        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$58,A10)</f>
-        <v>14</v>
+        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$60,A10)</f>
+        <v>16</v>
       </c>
       <c r="C10" s="14" t="n">
-        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$58,A10,รายละเอียดเทสเคส!$E$2:$E$58,"PASS")</f>
-        <v>14</v>
+        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$60,A10,รายละเอียดเทสเคส!$E$2:$E$60,"PASS")</f>
+        <v>16</v>
       </c>
       <c r="D10" s="14" t="n">
         <f aca="false">B10-C10</f>
@@ -2318,7 +2318,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>0.549</v>
+        <v>0.607</v>
       </c>
       <c r="G10" s="14" t="str">
         <f aca="false">IF(D10=0,"PASS","FAIL")</f>
@@ -2330,11 +2330,11 @@
         <v>35</v>
       </c>
       <c r="B11" s="18" t="n">
-        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$58,A11)</f>
+        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$60,A11)</f>
         <v>9</v>
       </c>
       <c r="C11" s="18" t="n">
-        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$58,A11,รายละเอียดเทสเคส!$E$2:$E$58,"PASS")</f>
+        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$60,A11,รายละเอียดเทสเคส!$E$2:$E$60,"PASS")</f>
         <v>9</v>
       </c>
       <c r="D11" s="18" t="n">
@@ -2346,7 +2346,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>0.063</v>
+        <v>0.059</v>
       </c>
       <c r="G11" s="18" t="str">
         <f aca="false">IF(D11=0,"PASS","FAIL")</f>
@@ -2358,11 +2358,11 @@
         <v>36</v>
       </c>
       <c r="B12" s="14" t="n">
-        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$58,A12)</f>
+        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$60,A12)</f>
         <v>7</v>
       </c>
       <c r="C12" s="14" t="n">
-        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$58,A12,รายละเอียดเทสเคส!$E$2:$E$58,"PASS")</f>
+        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$60,A12,รายละเอียดเทสเคส!$E$2:$E$60,"PASS")</f>
         <v>7</v>
       </c>
       <c r="D12" s="14" t="n">
@@ -2374,7 +2374,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="G12" s="14" t="str">
         <f aca="false">IF(D12=0,"PASS","FAIL")</f>
@@ -2386,11 +2386,11 @@
         <v>37</v>
       </c>
       <c r="B13" s="18" t="n">
-        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$58,A13)</f>
+        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$60,A13)</f>
         <v>7</v>
       </c>
       <c r="C13" s="18" t="n">
-        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$58,A13,รายละเอียดเทสเคส!$E$2:$E$58,"PASS")</f>
+        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$60,A13,รายละเอียดเทสเคส!$E$2:$E$60,"PASS")</f>
         <v>7</v>
       </c>
       <c r="D13" s="18" t="n">
@@ -2402,7 +2402,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="20" t="n">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
       <c r="G13" s="18" t="str">
         <f aca="false">IF(D13=0,"PASS","FAIL")</f>
@@ -2414,11 +2414,11 @@
         <v>38</v>
       </c>
       <c r="B14" s="14" t="n">
-        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$58,A14)</f>
+        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$60,A14)</f>
         <v>12</v>
       </c>
       <c r="C14" s="14" t="n">
-        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$58,A14,รายละเอียดเทสเคส!$E$2:$E$58,"PASS")</f>
+        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$60,A14,รายละเอียดเทสเคส!$E$2:$E$60,"PASS")</f>
         <v>12</v>
       </c>
       <c r="D14" s="14" t="n">
@@ -2430,7 +2430,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>0.026</v>
+        <v>0.023</v>
       </c>
       <c r="G14" s="14" t="str">
         <f aca="false">IF(D14=0,"PASS","FAIL")</f>
@@ -2442,11 +2442,11 @@
         <v>39</v>
       </c>
       <c r="B15" s="18" t="n">
-        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$58,A15)</f>
+        <f aca="false">COUNTIF(รายละเอียดเทสเคส!$B$2:$B$60,A15)</f>
         <v>8</v>
       </c>
       <c r="C15" s="18" t="n">
-        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$58,A15,รายละเอียดเทสเคส!$E$2:$E$58,"PASS")</f>
+        <f aca="false">COUNTIFS(รายละเอียดเทสเคส!$B$2:$B$60,A15,รายละเอียดเทสเคส!$E$2:$E$60,"PASS")</f>
         <v>8</v>
       </c>
       <c r="D15" s="18" t="n">
@@ -2458,7 +2458,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="20" t="n">
-        <v>0.04</v>
+        <v>0.018</v>
       </c>
       <c r="G15" s="18" t="str">
         <f aca="false">IF(D15=0,"PASS","FAIL")</f>
@@ -2471,11 +2471,11 @@
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">SUM(B10:B15)</f>
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C16" s="22" t="n">
         <f aca="false">SUM(C10:C15)</f>
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D16" s="22" t="n">
         <f aca="false">SUM(D10:D15)</f>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="F16" s="24" t="n">
         <f aca="false">SUM(F10:F15)</f>
-        <v>0.714</v>
+        <v>0.744</v>
       </c>
       <c r="G16" s="22" t="str">
         <f aca="false">IF(D16=0,"PASS","FAIL")</f>
@@ -2521,7 +2521,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3692,15 +3692,79 @@
         <v>55</v>
       </c>
     </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="18" t="inlineStr">
+        <is>
+          <t>TC-058</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>MemberServiceImplTest</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="D59" s="13" t="inlineStr">
+        <is>
+          <t>deleteMember_stillHasMembership_throws409</t>
+        </is>
+      </c>
+      <c r="E59" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F59" s="17" t="inlineStr">
+        <is>
+          <t>Error: Conflict (409)</t>
+        </is>
+      </c>
+    </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="29" t="s">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>TC-059</t>
+        </is>
+      </c>
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>MemberServiceImplTest</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="D60" s="13" t="inlineStr">
+        <is>
+          <t>deleteMember_stillHasTrainingSession_throws409</t>
+        </is>
+      </c>
+      <c r="E60" s="27" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="inlineStr">
+        <is>
+          <t>Error: Conflict (409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="29" t="s">
         <v>172</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F58"/>
+  <autoFilter ref="A1:F60"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E58" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E60" type="list">
       <formula1>"PASS,FAIL,SKIPPED"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>